<commit_message>
Import press release page as a content fragment reference
- New press-release import parser: releases with a content fragment import as a
  single Press Release block whose fragment field holds the fragment path (the
  article copy lives only in the fragment); 2015/11 re-imported
- Fragment field values stored in tools/cf-package/fragments/blue-september-2015.json
- Fragments folder policy allows the Press Release model (cq:allowedTemplates);
  package now updates the folder's jcr:content and the fragment only
- Site package uses the imported page as-is (no page rewrite)
- Packages bumped to 1.2.0 (vhi-ie-content-1.2.0.zip); 1.1.0 zips removed

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-press-release.report.xlsx
+++ b/tools/importer/reports/import-press-release.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="25">
   <si>
     <t>_reportFile</t>
   </si>
@@ -19,6 +19,12 @@
     <t>blocks</t>
   </si>
   <si>
+    <t>columns</t>
+  </si>
+  <si>
+    <t>panels</t>
+  </si>
+  <si>
     <t>path</t>
   </si>
   <si>
@@ -37,28 +43,49 @@
     <t>url</t>
   </si>
   <si>
+    <t>footer.report.json</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>footer</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>2026-09-29T11:58:36.364Z</t>
+  </si>
+  <si>
+    <t>https://www1.vhi.ie/about/media-releases-and-publications/2015/11</t>
+  </si>
+  <si>
+    <t>nav.report.json</t>
+  </si>
+  <si>
+    <t>nav</t>
+  </si>
+  <si>
+    <t>2026-09-29T11:58:25.956Z</t>
+  </si>
+  <si>
     <t>about/media-releases-and-publications/2015/11.report.json</t>
   </si>
   <si>
-    <t>[]</t>
+    <t>["press-release"]</t>
   </si>
   <si>
     <t>about/media-releases-and-publications/2015/11</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>press-release</t>
   </si>
   <si>
-    <t>2026-09-29T09:44:49.722Z</t>
+    <t>2026-09-29T13:30:29.702Z</t>
   </si>
   <si>
     <t>Blue September kicks off 2015 campaign revealing their new research on men's attitudes to their health</t>
-  </si>
-  <si>
-    <t>https://www1.vhi.ie/about/media-releases-and-publications/2015/11</t>
   </si>
 </sst>
 </file>
@@ -447,18 +474,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
-    <col min="2" max="2" width="8" customWidth="1"/>
-    <col min="3" max="3" width="47" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="8" width="50" customWidth="1"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="4" max="4" width="8" customWidth="1"/>
+    <col min="5" max="5" width="47" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="9" max="10" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -483,16 +511,22 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
       </c>
       <c r="D2" t="s">
         <v>11</v>
@@ -504,14 +538,84 @@
         <v>13</v>
       </c>
       <c r="G2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" t="s">
         <v>14</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
+      <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>